<commit_message>
Actualizar el cronograma al estado real del repo (semana 6)
Cierra las tareas 12 (Rayleigh-Sommerfeld 1D) y 14 (metrica SAM), y la 6
(interfaz comun), cuya nota decia que faltaba uniformar el retorno cuando
pipeline.propagar() ya lo hacia.

Desbloquea la tarea 3 (Figura 4): lo que faltaba eran justamente la metrica y
la referencia, y scripts/exactitud.py ya imprime la tabla. Queda graficarla.

Adelanta la 27 (validar con holograma simulado, semana 9) a En curso: la
validacion de extremo a extremo sobre DLHM-model ya esta hecha.

Anade tres tareas que no estaban en el plan y consumieron tiempo de la semana
6: el factor 2 del target USAF, K_fx/K_fy por eje y la separacion del paquete
por responsabilidad.

Avance global: 17 de 62 tareas, frente a 11 de 59 en la revision anterior.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/Cronograma_TG_DLHM.xlsx
+++ b/docs/Cronograma_TG_DLHM.xlsx
@@ -653,7 +653,7 @@
       </c>
       <c r="B9" s="23" t="inlineStr">
         <is>
-          <t>Jueves 13 de agosto de 2026 (semana 5)</t>
+          <t>Lunes 17 de agosto de 2026 (semana 6)</t>
         </is>
       </c>
       <c r="D9" s="26" t="n"/>
@@ -1391,7 +1391,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I64"/>
+  <dimension ref="A1:I67"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="14.4"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -1575,7 +1575,7 @@
       </c>
       <c r="I6" s="13" t="inlineStr">
         <is>
-          <t>Figura 4 = grafica de exactitud: SAM en dB vs z para ASM, BLAS, CRSD y MPASM. Bloqueada por la tarea 12 (referencia Rayleigh-Sommerfeld 1D) y la 14 (SAM del paper). Time_test.py del repo original SI corre en esta maquina.</t>
+          <t>DESBLOQUEADA: ya estan la metrica SAM (tarea 14) y la referencia R-S (tarea 12), que eran lo que faltaba. scripts/exactitud.py ya imprime la tabla: MPASM se mantiene entre 31 y 48 dB de z=500 a 200000 mm, FFT-ASM cae de 40 a -1.85 dB y BL-ASM se degrada y luego se recupera. Falta graficarlo contra z.</t>
         </is>
       </c>
     </row>
@@ -1690,7 +1690,7 @@
       </c>
       <c r="G9" s="12" t="inlineStr">
         <is>
-          <t>En curso</t>
+          <t>Hecho</t>
         </is>
       </c>
       <c r="H9" s="12" t="inlineStr">
@@ -1700,7 +1700,7 @@
       </c>
       <c r="I9" s="13" t="inlineStr">
         <is>
-          <t>Interfaz comun ya operativa: (U0, delta, lamb, z, device, dtype) en mpasm/fft_asm/blas. Falta uniformar el retorno: mpasm devuelve (campo, Kf) y los otros solo el campo.</t>
+          <t>Hecha. La interfaz comun es pipeline.propagar(U0, delta, lamb, z, metodo, pad, device, dtype) -&gt; (campo, info), uniforme para los tres metodos. Las funciones de bajo nivel conservan su retorno propio a proposito: mpasm devuelve Kf porque es un resultado del metodo, no un detalle de implementacion.</t>
         </is>
       </c>
     </row>
@@ -1948,7 +1948,7 @@
       </c>
       <c r="G15" s="12" t="inlineStr">
         <is>
-          <t>En curso</t>
+          <t>Hecho</t>
         </is>
       </c>
       <c r="H15" s="12" t="inlineStr">
@@ -1958,7 +1958,7 @@
       </c>
       <c r="I15" s="13" t="inlineStr">
         <is>
-          <t>La RS completa de pyLHM (rayleigh1Free) ya corre: el parche 1 de parchar_referencias.py arreglo el dtype='complex_' que la rompia con NumPy 2. Decidir si la tarea se reduce a contrastar contra ella o si hace falta una implementacion propia 1D.</t>
+          <t>Hecha. CamposT/referencias.py, rs1_radial(): R-S I exacta reducida a 1-D por simetria circular (el paper dice que reduce el calculo 2-D a 1-D pero no como; es reescribir la integral en polares, sin aproximar). O(N_rho^2 N_phi) en vez de O(N^4): la fuerza bruta de pyLHM tardaria 1-2 h en la malla de la Tabla 1. Contrastada contra esa fuerza bruta y 19x mas exacta que ella (1.0e-3 frente a 1.9e-2 contra la analitica). No es paraxial, asi que su diferencia con gauss_analytic mide la paraxialidad. 11 tests, mutacion 8/8.</t>
         </is>
       </c>
     </row>
@@ -2001,7 +2001,7 @@
       </c>
       <c r="I16" s="13" t="inlineStr">
         <is>
-          <t>Verificacion hecha en tres frentes: tests/test_propagadores.py exige a MPASM (s=4, Kf auto) RMS &lt; 1e-3 contra gauss_analytic a z = 12000 y 80000 mm; contraste_referencias.py usa el gaussiano como arbitro frente a pyDHM; figura_escenario.py confirma el factor geometrico w0*(R+z)/R. Falta el entregable: las curvas de error graficadas.</t>
+          <t>Verificacion hecha y ampliada: ahora hay DOS referencias independientes (gauss_analytic, paraxial, y rs1_radial, no paraxial) y la metrica correcta. scripts/exactitud.py imprime la tabla SAM vs z. Falta solo el entregable: graficar las curvas de error.</t>
         </is>
       </c>
     </row>
@@ -2034,7 +2034,7 @@
       </c>
       <c r="G17" s="12" t="inlineStr">
         <is>
-          <t>En curso</t>
+          <t>Hecho</t>
         </is>
       </c>
       <c r="H17" s="12" t="inlineStr">
@@ -2044,7 +2044,7 @@
       </c>
       <c r="I17" s="13" t="inlineStr">
         <is>
-          <t>DEFINICION ENCONTRADA en el paper, Ecs. (15)-(16): SAM = 10*lg[ integral I / integral |I - alfa*I_ref| ], alfa = integral I*conj(I_ref) / integral I_ref. Sobre INTENSIDADES y en dB (mas alto = mejor). sam() en propagadores.py SIGUE siendo un RMS de amplitudes normalizadas: mide otra cosa. Nada la bloquea; bloquea a la tarea 3 (Figura 4).</t>
+          <t>Hecha. CamposT/metricas.py, sam(). ERRATA ENCONTRADA en la Ec. (16): el denominador impreso es integral I_ref y tiene que ser integral I_ref^2. Con la impresa, un campo identico a su referencia da 0.365 dB en vez de infinito y el SAM queda bajo 2.5 dB para todo, o sea que el paper no habria podido generar su propia Figura 4. Segunda errata, tras el A^2*B de la Ec. (14). sam(formula='literal') reproduce la impresa. 11 tests, mutacion 6/6.</t>
         </is>
       </c>
     </row>
@@ -2555,7 +2555,7 @@
       </c>
       <c r="G30" s="12" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>En curso</t>
         </is>
       </c>
       <c r="H30" s="12" t="inlineStr">
@@ -2563,7 +2563,11 @@
           <t>18/09/2026</t>
         </is>
       </c>
-      <c r="I30" s="13" t="n"/>
+      <c r="I30" s="13" t="inlineStr">
+        <is>
+          <t>ADELANTADA (era semana 9). Validacion de extremo a extremo sobre DLHM-model: holograma simulado con verdad-terreno conocida, retropropagado con MPASM. La fase reconstruida a la distancia nominal devuelve el target con los grupos de barras USAF y sus numeros legibles, sin ajustar parametros. Dos lecciones: el caso cae FUERA del rango de FFT-ASM (z_lim = 6.6 mm frente a z = 24 mm), y el criterio de autofoco depende del tipo de objeto (en fase hay que MINIMIZAR la varianza de amplitud, no maximizar nitidez). Falta versionarlo como scripts/reconstruccion_dlhm.py.</t>
+        </is>
+      </c>
     </row>
     <row r="31" ht="25.5" customHeight="1">
       <c r="A31" s="12" t="n">
@@ -3829,8 +3833,137 @@
         </is>
       </c>
     </row>
+    <row r="63">
+      <c r="A63" s="12" t="n">
+        <v>60</v>
+      </c>
+      <c r="B63" s="12" t="n">
+        <v>6</v>
+      </c>
+      <c r="C63" s="12" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
+      <c r="D63" s="13" t="inlineStr">
+        <is>
+          <t>Corregir el factor 2 en la conversion del target USAF a lp/mm</t>
+        </is>
+      </c>
+      <c r="E63" s="13" t="inlineStr">
+        <is>
+          <t>Geometria contrastada contra la imagen</t>
+        </is>
+      </c>
+      <c r="F63" s="12" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="G63" s="12" t="inlineStr">
+        <is>
+          <t>Hecho</t>
+        </is>
+      </c>
+      <c r="H63" s="12" t="inlineStr">
+        <is>
+          <t>21/08/2026</t>
+        </is>
+      </c>
+      <c r="I63" s="13" t="inlineStr">
+        <is>
+          <t>periodos_usaf devolvia el ancho de barra llamandolo periodo. Un par de lineas es barra+hueco = 2b, asi que toda cifra de resolucion habria salido con factor 2. Alimenta directamente la tarea 40. Ahora anchos_barra_usaf / periodos_usaf / lineas_por_mm_usaf salen de una sola fuente, la misma con la que dibuja usaf_like.</t>
+        </is>
+      </c>
+    </row>
     <row r="64">
-      <c r="D64" s="21" t="inlineStr">
+      <c r="A64" s="12" t="n">
+        <v>61</v>
+      </c>
+      <c r="B64" s="12" t="n">
+        <v>6</v>
+      </c>
+      <c r="C64" s="12" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
+      <c r="D64" s="13" t="inlineStr">
+        <is>
+          <t>Calcular K_fx y K_fy por eje para campos no cuadrados</t>
+        </is>
+      </c>
+      <c r="E64" s="13" t="inlineStr">
+        <is>
+          <t>Propagador correcto en malla rectangular</t>
+        </is>
+      </c>
+      <c r="F64" s="12" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="G64" s="12" t="inlineStr">
+        <is>
+          <t>Hecho</t>
+        </is>
+      </c>
+      <c r="H64" s="12" t="inlineStr">
+        <is>
+          <t>21/08/2026</t>
+        </is>
+      </c>
+      <c r="I64" s="13" t="inlineStr">
+        <is>
+          <t>La Tabla 1 los lista por separado y mpasm usaba uno solo. Kf va como ~1/sqrt(N), asi que el eje corto quedaba submuestreado en silencio. Con un target USAF en malla 64x128 el error es 5x a 63x mayor; con un gaussiano NO se aprecia, porque hace falta contenido cerca del limite de banda para que aparezca aliasing. Los sensores de DLHM no son cuadrados: esto habria aparecido en la semana 11.</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="12" t="n">
+        <v>62</v>
+      </c>
+      <c r="B65" s="12" t="n">
+        <v>6</v>
+      </c>
+      <c r="C65" s="12" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
+      <c r="D65" s="13" t="inlineStr">
+        <is>
+          <t>Separar el paquete por responsabilidad (referencias, metricas, pipeline)</t>
+        </is>
+      </c>
+      <c r="E65" s="13" t="inlineStr">
+        <is>
+          <t>Paquete navegable</t>
+        </is>
+      </c>
+      <c r="F65" s="12" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="G65" s="12" t="inlineStr">
+        <is>
+          <t>Hecho</t>
+        </is>
+      </c>
+      <c r="H65" s="12" t="inlineStr">
+        <is>
+          <t>21/08/2026</t>
+        </is>
+      </c>
+      <c r="I65" s="13" t="inlineStr">
+        <is>
+          <t>propagadores.py habia llegado a 539 lineas con cuatro asuntos dentro y campos.py mezclaba construir el campo con propagarlo y guardarlo. Ahora seis modulos de un tema cada uno, ninguno de mas de 235 lineas: campos, propagadores, referencias, metricas, pipeline y backend. 158 tests en verde antes y despues: el comportamiento no cambio.</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="D67" t="inlineStr">
         <is>
           <t>Ejemplo de uso: 'En curso' mientras trabajas la tarea, 'Bloqueado' si depende de un tercero (laboratorio, asesor).</t>
         </is>

</xml_diff>

<commit_message>
Cronograma: anadir la tarea 74 y extender el autofiltro
La tarea 74 -soporte de GPU en los cuatro mi_prueba_*- entra retroactiva, con
los numeros medidos en la nota, como el resto. Semana Receso y fase F1, la
misma que la tarea 57, que es el otro trabajo del eje CPU/GPU.

El avance queda en 38 de 74 tareas hechas, 51.4 %, con F1 en 31 de 32.

Y un arreglo del propio archivo: el autofiltro se habia quedado en A3:I74
cuando se anadieron las tareas 71 a 73, asi que esas tres filas quedaban fuera
del filtro. Va a A3:I77. La validacion de Estado y el formato condicional ya
cubrian hasta la fila 200 y no hizo falta tocarlos.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/Cronograma_TG_DLHM.xlsx
+++ b/docs/Cronograma_TG_DLHM.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" firstSheet="0" activeTab="2" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="Resumen" sheetId="1" state="visible" r:id="rId1"/>
@@ -12,7 +12,7 @@
     <sheet name="Hitos" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Tareas'!$A$3:$I$62</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Tareas'!$A$3:$I$77</definedName>
   </definedNames>
   <calcPr calcId="191029" fullCalcOnLoad="1" iterateDelta="0.0001"/>
 </workbook>
@@ -23,7 +23,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="9">
+  <fonts count="7">
     <font>
       <name val="Calibri"/>
       <charset val="1"/>
@@ -52,11 +52,6 @@
     <font>
       <name val="Arial"/>
       <charset val="1"/>
-      <sz val="9"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <charset val="1"/>
       <b val="1"/>
       <color rgb="FF1F3864"/>
       <sz val="11"/>
@@ -67,13 +62,6 @@
       <b val="1"/>
       <color rgb="FFFFFFFF"/>
       <sz val="10"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <charset val="1"/>
-      <i val="1"/>
-      <color rgb="FF808080"/>
-      <sz val="9"/>
     </font>
     <font>
       <name val="Arial"/>
@@ -114,7 +102,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="5">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -137,61 +125,28 @@
       </bottom>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color rgb="FFBFBFBF"/>
-      </left>
-      <right/>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FFBFBFBF"/>
-      </left>
-      <right style="thin">
-        <color rgb="FFBFBFBF"/>
-      </right>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FFBFBFBF"/>
-      </left>
-      <right style="thin">
-        <color rgb="FFBFBFBF"/>
-      </right>
-      <top/>
-      <bottom style="thin">
-        <color rgb="FFBFBFBF"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="29">
+  <cellXfs count="25">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="164" fontId="2" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -230,18 +185,10 @@
     <xf numFmtId="9" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -545,20 +492,19 @@
   <dimension ref="A1:D23"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="14.4"/>
   <cols>
-    <col width="38" customWidth="1" min="1" max="1"/>
-    <col width="18" customWidth="1" min="2" max="2"/>
-    <col width="42.5546875" customWidth="1" min="3" max="3"/>
-    <col width="60" customWidth="1" min="4" max="4"/>
+    <col width="38" customWidth="1" style="22" min="1" max="1"/>
+    <col width="18" customWidth="1" style="22" min="2" max="2"/>
+    <col width="42.5546875" customWidth="1" style="22" min="3" max="3"/>
   </cols>
   <sheetData>
-    <row r="1" ht="21.75" customHeight="1">
-      <c r="A1" s="22" t="inlineStr">
+    <row r="1" ht="21.75" customHeight="1" s="22">
+      <c r="A1" s="21" t="inlineStr">
         <is>
           <t>Trabajo de grado 2026-2 - Propagadores con control de muestreo en DLHM</t>
         </is>
       </c>
     </row>
-    <row r="3" ht="15" customHeight="1">
+    <row r="3" ht="15" customHeight="1" s="22">
       <c r="A3" s="2" t="inlineStr">
         <is>
           <t>Estudiante</t>
@@ -569,7 +515,7 @@
           <t>Camilo Rodriguez Londono</t>
         </is>
       </c>
-      <c r="D3" s="24" t="inlineStr">
+      <c r="D3" t="inlineStr">
         <is>
           <t>COMO USAR ESTE ARCHIVO
 1. La unica columna que se edita a diario es 'Estado' en la hoja Tareas (lista desplegable: Pendiente / En curso / Hecho / Bloqueado).
@@ -591,7 +537,6 @@
           <t>Carlos Alejandro Trujillo Anaya, PhD</t>
         </is>
       </c>
-      <c r="D4" s="26" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -604,7 +549,6 @@
           <t>Ingenieria Fisica - Universidad EAFIT</t>
         </is>
       </c>
-      <c r="D5" s="26" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -617,7 +561,6 @@
           <t>Opcion 2 (grados de diciembre, sin mencion de honor)</t>
         </is>
       </c>
-      <c r="D6" s="26" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -630,7 +573,6 @@
           <t>Viernes 30 de octubre de 2026 (semana 15)</t>
         </is>
       </c>
-      <c r="D7" s="26" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -643,7 +585,6 @@
           <t>Hasta el viernes 20 de noviembre de 2026</t>
         </is>
       </c>
-      <c r="D8" s="26" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -653,10 +594,9 @@
       </c>
       <c r="B9" s="23" t="inlineStr">
         <is>
-          <t>Domingo 23 de agosto de 2026 (fin de semana 6)</t>
-        </is>
-      </c>
-      <c r="D9" s="26" t="n"/>
+          <t>Martes 1 de septiembre de 2026 (semana 8, dia 2)</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
@@ -664,7 +604,6 @@
           <t>AVANCE GLOBAL</t>
         </is>
       </c>
-      <c r="D10" s="26" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="23" t="inlineStr">
@@ -676,7 +615,6 @@
         <f>COUNTA(Tareas!$A$4:$A$200)</f>
         <v/>
       </c>
-      <c r="D11" s="26" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="23" t="inlineStr">
@@ -688,7 +626,6 @@
         <f>COUNTIF(Tareas!$G$4:$G$200,"Hecho")</f>
         <v/>
       </c>
-      <c r="D12" s="26" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="23" t="inlineStr">
@@ -700,7 +637,6 @@
         <f>COUNTIF(Tareas!$G$4:$G$200,"En curso")</f>
         <v/>
       </c>
-      <c r="D13" s="26" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="23" t="inlineStr">
@@ -712,7 +648,6 @@
         <f>COUNTIF(Tareas!$G$4:$G$200,"Bloqueado")</f>
         <v/>
       </c>
-      <c r="D14" s="26" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="23" t="inlineStr">
@@ -724,10 +659,6 @@
         <f>IFERROR(B12/B11,0)</f>
         <v/>
       </c>
-      <c r="D15" s="26" t="n"/>
-    </row>
-    <row r="16">
-      <c r="D16" s="26" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
@@ -735,7 +666,6 @@
           <t>AVANCE POR FASE</t>
         </is>
       </c>
-      <c r="D17" s="26" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="6" t="inlineStr">
@@ -753,7 +683,6 @@
           <t>Hechas</t>
         </is>
       </c>
-      <c r="D18" s="26" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="23" t="inlineStr">
@@ -769,7 +698,6 @@
         <f>COUNTIFS(Tareas!$C$4:$C$200,"F1",Tareas!$G$4:$G$200,"Hecho")</f>
         <v/>
       </c>
-      <c r="D19" s="26" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="23" t="inlineStr">
@@ -785,7 +713,6 @@
         <f>COUNTIFS(Tareas!$C$4:$C$200,"F2",Tareas!$G$4:$G$200,"Hecho")</f>
         <v/>
       </c>
-      <c r="D20" s="26" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="23" t="inlineStr">
@@ -801,7 +728,6 @@
         <f>COUNTIFS(Tareas!$C$4:$C$200,"F3",Tareas!$G$4:$G$200,"Hecho")</f>
         <v/>
       </c>
-      <c r="D21" s="26" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="23" t="inlineStr">
@@ -817,7 +743,6 @@
         <f>COUNTIFS(Tareas!$C$4:$C$200,"F4",Tareas!$G$4:$G$200,"Hecho")</f>
         <v/>
       </c>
-      <c r="D22" s="26" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="23" t="inlineStr">
@@ -833,15 +758,13 @@
         <f>COUNTIFS(Tareas!$C$4:$C$200,"HITO",Tareas!$G$4:$G$200,"Hecho")</f>
         <v/>
       </c>
-      <c r="D23" s="27" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="9">
-    <mergeCell ref="A1:D1"/>
+  <mergeCells count="8">
     <mergeCell ref="B6:C6"/>
     <mergeCell ref="B7:C7"/>
+    <mergeCell ref="A1:C1"/>
     <mergeCell ref="B3:C3"/>
-    <mergeCell ref="D3:D23"/>
     <mergeCell ref="B5:C5"/>
     <mergeCell ref="B9:C9"/>
     <mergeCell ref="B8:C8"/>
@@ -861,24 +784,24 @@
   <dimension ref="A1:H16"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="14.4"/>
   <cols>
-    <col width="10" customWidth="1" min="1" max="1"/>
-    <col width="18" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="44" customWidth="1" min="4" max="4"/>
-    <col width="40" customWidth="1" min="5" max="5"/>
-    <col width="32" customWidth="1" min="6" max="6"/>
-    <col width="10" customWidth="1" min="7" max="7"/>
-    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="10" customWidth="1" style="22" min="1" max="1"/>
+    <col width="18" customWidth="1" style="22" min="2" max="2"/>
+    <col width="12" customWidth="1" style="22" min="3" max="3"/>
+    <col width="44" customWidth="1" style="22" min="4" max="4"/>
+    <col width="40" customWidth="1" style="22" min="5" max="5"/>
+    <col width="32" customWidth="1" style="22" min="6" max="6"/>
+    <col width="10" customWidth="1" style="22" min="7" max="7"/>
+    <col width="12" customWidth="1" style="22" min="8" max="8"/>
   </cols>
   <sheetData>
-    <row r="1" ht="21.75" customHeight="1">
-      <c r="A1" s="22" t="inlineStr">
+    <row r="1" ht="21.75" customHeight="1" s="22">
+      <c r="A1" s="21" t="inlineStr">
         <is>
           <t>Cronograma semana a semana</t>
         </is>
       </c>
     </row>
-    <row r="3" ht="30" customHeight="1">
+    <row r="3" ht="30" customHeight="1" s="22">
       <c r="A3" s="8" t="inlineStr">
         <is>
           <t>Semana</t>
@@ -920,7 +843,7 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="33.75" customHeight="1">
+    <row r="4" ht="33.75" customHeight="1" s="22">
       <c r="A4" s="9" t="n">
         <v>4</v>
       </c>
@@ -954,7 +877,7 @@
         <v/>
       </c>
     </row>
-    <row r="5" ht="33.75" customHeight="1">
+    <row r="5" ht="33.75" customHeight="1" s="22">
       <c r="A5" s="12" t="n">
         <v>5</v>
       </c>
@@ -988,7 +911,7 @@
         <v/>
       </c>
     </row>
-    <row r="6" ht="33.75" customHeight="1">
+    <row r="6" ht="33.75" customHeight="1" s="22">
       <c r="A6" s="9" t="n">
         <v>6</v>
       </c>
@@ -1022,7 +945,7 @@
         <v/>
       </c>
     </row>
-    <row r="7" ht="33.75" customHeight="1">
+    <row r="7" ht="33.75" customHeight="1" s="22">
       <c r="A7" s="12" t="n">
         <v>7</v>
       </c>
@@ -1056,7 +979,7 @@
         <v/>
       </c>
     </row>
-    <row r="8" ht="33.75" customHeight="1">
+    <row r="8" ht="33.75" customHeight="1" s="22">
       <c r="A8" s="15" t="n">
         <v>8</v>
       </c>
@@ -1094,7 +1017,7 @@
         <v/>
       </c>
     </row>
-    <row r="9" ht="33.75" customHeight="1">
+    <row r="9" ht="33.75" customHeight="1" s="22">
       <c r="A9" s="18" t="inlineStr">
         <is>
           <t>Receso</t>
@@ -1130,7 +1053,7 @@
         <v/>
       </c>
     </row>
-    <row r="10" ht="33.75" customHeight="1">
+    <row r="10" ht="33.75" customHeight="1" s="22">
       <c r="A10" s="9" t="n">
         <v>9</v>
       </c>
@@ -1164,7 +1087,7 @@
         <v/>
       </c>
     </row>
-    <row r="11" ht="33.75" customHeight="1">
+    <row r="11" ht="33.75" customHeight="1" s="22">
       <c r="A11" s="12" t="n">
         <v>10</v>
       </c>
@@ -1198,7 +1121,7 @@
         <v/>
       </c>
     </row>
-    <row r="12" ht="33.75" customHeight="1">
+    <row r="12" ht="33.75" customHeight="1" s="22">
       <c r="A12" s="9" t="n">
         <v>11</v>
       </c>
@@ -1232,7 +1155,7 @@
         <v/>
       </c>
     </row>
-    <row r="13" ht="33.75" customHeight="1">
+    <row r="13" ht="33.75" customHeight="1" s="22">
       <c r="A13" s="12" t="n">
         <v>12</v>
       </c>
@@ -1266,7 +1189,7 @@
         <v/>
       </c>
     </row>
-    <row r="14" ht="33.75" customHeight="1">
+    <row r="14" ht="33.75" customHeight="1" s="22">
       <c r="A14" s="9" t="n">
         <v>13</v>
       </c>
@@ -1300,7 +1223,7 @@
         <v/>
       </c>
     </row>
-    <row r="15" ht="33.75" customHeight="1">
+    <row r="15" ht="33.75" customHeight="1" s="22">
       <c r="A15" s="15" t="n">
         <v>14</v>
       </c>
@@ -1338,7 +1261,7 @@
         <v/>
       </c>
     </row>
-    <row r="16" ht="33.75" customHeight="1">
+    <row r="16" ht="33.75" customHeight="1" s="22">
       <c r="A16" s="15" t="n">
         <v>15</v>
       </c>
@@ -1391,27 +1314,27 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I70"/>
+  <dimension ref="A1:I77"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="14.4"/>
   <cols>
-    <col width="7" customWidth="1" min="1" max="1"/>
-    <col width="10" customWidth="1" min="2" max="2"/>
-    <col width="9" customWidth="1" min="3" max="3"/>
-    <col width="62" customWidth="1" min="4" max="4"/>
-    <col width="30" customWidth="1" min="5" max="5"/>
-    <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="14" customWidth="1" min="7" max="8"/>
-    <col width="34" customWidth="1" min="9" max="9"/>
+    <col width="7" customWidth="1" style="22" min="1" max="1"/>
+    <col width="10" customWidth="1" style="22" min="2" max="2"/>
+    <col width="9" customWidth="1" style="22" min="3" max="3"/>
+    <col width="62" customWidth="1" style="22" min="4" max="4"/>
+    <col width="30" customWidth="1" style="22" min="5" max="5"/>
+    <col width="12" customWidth="1" style="22" min="6" max="6"/>
+    <col width="14" customWidth="1" style="22" min="7" max="8"/>
+    <col width="34" customWidth="1" style="22" min="9" max="9"/>
   </cols>
   <sheetData>
-    <row r="1" ht="21.75" customHeight="1">
-      <c r="A1" s="22" t="inlineStr">
+    <row r="1" ht="21.75" customHeight="1" s="22">
+      <c r="A1" s="21" t="inlineStr">
         <is>
           <t>Lista de tareas - editar solo la columna Estado</t>
         </is>
       </c>
     </row>
-    <row r="3" ht="30" customHeight="1">
+    <row r="3" ht="30" customHeight="1" s="22">
       <c r="A3" s="8" t="inlineStr">
         <is>
           <t>ID</t>
@@ -1458,7 +1381,7 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="25.5" customHeight="1">
+    <row r="4" ht="25.5" customHeight="1" s="22">
       <c r="A4" s="12" t="n">
         <v>1</v>
       </c>
@@ -1487,7 +1410,7 @@
       </c>
       <c r="G4" s="12" t="inlineStr">
         <is>
-          <t>En curso</t>
+          <t>Hecho</t>
         </is>
       </c>
       <c r="H4" s="12" t="inlineStr">
@@ -1497,11 +1420,11 @@
       </c>
       <c r="I4" s="13" t="inlineStr">
         <is>
-          <t>Sigue abierta desde la semana 4, vencio el 07/08. O se cierra, o se convierte en lista concreta de ajustes: es lo que se presenta como respuesta a la sustentacion en el informe de avance 1.</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="25.5" customHeight="1">
+          <t>CERRADA el 31/08. Los ajustes acordados en la sustentacion se responden en el material del avance 1. Estuvo abierta 24 dias mas alla de su fecha (07/08): es la tarea que mas tiempo llevo sin cerrar.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="25.5" customHeight="1" s="22">
       <c r="A5" s="12" t="n">
         <v>2</v>
       </c>
@@ -1540,7 +1463,7 @@
       </c>
       <c r="I5" s="13" t="n"/>
     </row>
-    <row r="6" ht="25.5" customHeight="1">
+    <row r="6" ht="25.5" customHeight="1" s="22">
       <c r="A6" s="12" t="n">
         <v>3</v>
       </c>
@@ -1583,7 +1506,7 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="25.5" customHeight="1">
+    <row r="7" ht="25.5" customHeight="1" s="22">
       <c r="A7" s="12" t="n">
         <v>4</v>
       </c>
@@ -1626,7 +1549,7 @@
         </is>
       </c>
     </row>
-    <row r="8" ht="25.5" customHeight="1">
+    <row r="8" ht="25.5" customHeight="1" s="22">
       <c r="A8" s="12" t="n">
         <v>5</v>
       </c>
@@ -1665,7 +1588,7 @@
       </c>
       <c r="I8" s="13" t="n"/>
     </row>
-    <row r="9" ht="25.5" customHeight="1">
+    <row r="9" ht="25.5" customHeight="1" s="22">
       <c r="A9" s="12" t="n">
         <v>6</v>
       </c>
@@ -1708,7 +1631,7 @@
         </is>
       </c>
     </row>
-    <row r="10" ht="25.5" customHeight="1">
+    <row r="10" ht="25.5" customHeight="1" s="22">
       <c r="A10" s="12" t="n">
         <v>7</v>
       </c>
@@ -1747,11 +1670,11 @@
       </c>
       <c r="I10" s="13" t="inlineStr">
         <is>
-          <t>CamposT/propagadores.py, fft_asm(). Revisado el 23/08 (commit c5fd678): aplica la transferencia in situ en vez de materializar H y multiplicar, que pedia dos arrays del tamano del plano de mas. Bit a bit identico, +4 % CPU y +7.6 % GPU.</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="25.5" customHeight="1">
+          <t>CamposT/propagadores.py, fft_asm(). Revisado el 23/08 (commit c5fd678): aplica la transferencia in situ en vez de materializar H y multiplicar, que pedia dos arrays del tamano del plano de mas. Bit a bit identico, +4 % CPU y +7.6 % GPU. Corregido otra vez en la semana 7: ver tarea 66 (la rejilla de frecuencias estaba medio paso corrida en malla impar).</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="25.5" customHeight="1" s="22">
       <c r="A11" s="12" t="n">
         <v>8</v>
       </c>
@@ -1790,11 +1713,11 @@
       </c>
       <c r="I11" s="13" t="inlineStr">
         <is>
-          <t>CamposT/propagadores.py, blas() - Matsushima &amp; Shimobaba (2009). Revisado el 23/08 (commit c5fd678): el limite de banda es un rectangulo centrado, asi que se anulan las cuatro bandas de fuera por rodajas en vez de construir H, dos meshgrid y una mascara. Bit a bit identico, +8.3 % CPU y +17.4 % GPU, y 1.6 GB menos de picos sobre una malla de 6000x8000.</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="25.5" customHeight="1">
+          <t>CamposT/propagadores.py, blas() - Matsushima &amp; Shimobaba (2009). Revisado el 23/08 (commit c5fd678): el limite de banda es un rectangulo centrado, asi que se anulan las cuatro bandas de fuera por rodajas en vez de construir H, dos meshgrid y una mascara. Bit a bit identico, +8.3 % CPU y +17.4 % GPU, y 1.6 GB menos de picos sobre una malla de 6000x8000. Corregido otra vez en la semana 7: ver tarea 66 (la misma rejilla medio paso corrida que fft_asm).</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="25.5" customHeight="1" s="22">
       <c r="A12" s="12" t="n">
         <v>9</v>
       </c>
@@ -1833,11 +1756,11 @@
       </c>
       <c r="I12" s="13" t="inlineStr">
         <is>
-          <t>tests/test_propagadores.py + tests/conftest.py, 119 casos, verde. Cubre z=0, energia, reversibilidad, MPASM con Kf&gt;1, paridad CPU/GPU, kf_auto y la funcion de transferencia. Validada por mutacion: 6 bugs inyectados, 6 detectados. Correr con: python -m pytest Al 23/08 la suite va por 186 casos en verde, 19 de ellos de retropropagacion (tarea 64). Al 23/08 la suite va por 213 casos en verde. Se suma tests/test_pipeline.py (commit c5fd678): pipeline.py es la puerta de entrada del paquete y no tenia suite propia, solo se comprobaba de refilon.</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="25.5" customHeight="1">
+          <t>tests/test_propagadores.py + tests/conftest.py. Cubre z=0, energia, reversibilidad, MPASM con Kf&gt;1, paridad CPU/GPU, kf_auto y la funcion de transferencia. Validada por mutacion: 6 bugs inyectados, 6 detectados. Correr con: python -m pytest La suite fue creciendo con el paquete: 119 casos al crearse, 186 y 213 el 23/08 (retropropagacion y pipeline). AL 31/08 VA POR 299 CASOS EN VERDE en 56 s: los nuevos vienen de la rejilla centrada (16, tarea 66), el modo mixto, las fases de la retropropagacion, la nitidez, el pico de foco y la intensidad sin gamma. CERRADO el 01/09 lo de tests/mi_test.py (tarea 72): no costaba 12.2 s, COLGABA la recoleccion. Movido a scripts/, la suite pasa de 56 s a 38.29 s con los mismos 299 casos en verde.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="25.5" customHeight="1" s="22">
       <c r="A13" s="12" t="n">
         <v>10</v>
       </c>
@@ -1880,7 +1803,7 @@
         </is>
       </c>
     </row>
-    <row r="14" ht="25.5" customHeight="1">
+    <row r="14" ht="25.5" customHeight="1" s="22">
       <c r="A14" s="12" t="n">
         <v>11</v>
       </c>
@@ -1923,7 +1846,7 @@
         </is>
       </c>
     </row>
-    <row r="15" ht="25.5" customHeight="1">
+    <row r="15" ht="25.5" customHeight="1" s="22">
       <c r="A15" s="12" t="n">
         <v>12</v>
       </c>
@@ -1966,7 +1889,7 @@
         </is>
       </c>
     </row>
-    <row r="16" ht="25.5" customHeight="1">
+    <row r="16" ht="25.5" customHeight="1" s="22">
       <c r="A16" s="12" t="n">
         <v>13</v>
       </c>
@@ -2009,7 +1932,7 @@
         </is>
       </c>
     </row>
-    <row r="17" ht="25.5" customHeight="1">
+    <row r="17" ht="25.5" customHeight="1" s="22">
       <c r="A17" s="12" t="n">
         <v>14</v>
       </c>
@@ -2052,7 +1975,7 @@
         </is>
       </c>
     </row>
-    <row r="18" ht="25.5" customHeight="1">
+    <row r="18" ht="25.5" customHeight="1" s="22">
       <c r="A18" s="12" t="n">
         <v>15</v>
       </c>
@@ -2091,11 +2014,11 @@
       </c>
       <c r="I18" s="13" t="inlineStr">
         <is>
-          <t>Sin empezar, vencida el 21/08. Es el insumo directo de las diapositivas del avance 1 (tarea 19): el material ya esta en el README y en los docstrings del paquete, falta pasarlo a texto de tesis.</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="25.5" customHeight="1">
+          <t>SIN EMPEZAR el 31/08, diez dias despues de vencer. Las diapositivas del avance 1 salieron sin ella. El material esta escrito pero disperso -el README, los docstrings del paquete y las notas de este cronograma-: falta pasarlo a prosa de tesis, y a partir de hoy compite con la Fase 2. Es la primera deuda de escritura del proyecto. AL 01/09 SIGUE SIN EMPEZAR y queda fuera del foco de la semana 8 y del receso, que se dedican a la tarea 17, a la Fase 2 (24-26) y a la limpieza del repo. Se arrastra a la semana 9, donde ya compite con F2. Es la segunda vez que se aplaza.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="25.5" customHeight="1" s="22">
       <c r="A19" s="12" t="n">
         <v>16</v>
       </c>
@@ -2124,7 +2047,7 @@
       </c>
       <c r="G19" s="12" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Hecho</t>
         </is>
       </c>
       <c r="H19" s="12" t="inlineStr">
@@ -2132,9 +2055,13 @@
           <t>28/08/2026</t>
         </is>
       </c>
-      <c r="I19" s="13" t="n"/>
-    </row>
-    <row r="20" ht="25.5" customHeight="1">
+      <c r="I19" s="13" t="inlineStr">
+        <is>
+          <t>Hecha en la semana 7. Queda pendiente lo que tenia que salir de ella: los parametros reales del montaje (tarea 17).</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="25.5" customHeight="1" s="22">
       <c r="A20" s="12" t="n">
         <v>17</v>
       </c>
@@ -2173,11 +2100,11 @@
       </c>
       <c r="I20" s="13" t="inlineStr">
         <is>
-          <t>Sin estos parametros la Fase 2 (semanas 9 y 10) arranca simulando sobre valores inventados. Es la dependencia mas critica de la semana 7.</t>
-        </is>
-      </c>
-    </row>
-    <row r="21" ht="25.5" customHeight="1">
+          <t>VENCIDA el 28/08 y abierta al 31/08. Es la dependencia mas critica del cronograma: la Fase 2 arranca el 14/09 -dos semanas, con el receso de por medio- y sin lambda, pitch, sensor, L, z y NA reales el barrido de la tarea 30 se corre sobre valores inventados y hay que repetirlo. El acceso al montaje ya no es el bloqueo: la sesion de familiarizacion (tarea 16) y la reserva de laboratorio (tarea 18) estan hechas. AL 01/09 ES EL FOCO DE LA SEMANA 8: quedan cuatro dias habiles (1-4 sep) antes del receso, y despues del receso solo queda la semana del 14/09, que es cuando arranca la Fase 2 que depende de estos numeros. Al 01/09 su entregable esta PREPARADO Y VACIO (tarea 73): docs/hoja_parametros_montaje.md es el checklist que se lleva al laboratorio y CamposT/montaje.py el destino de los numeros. Faltan los 15 valores; cualquier cuenta que use uno de ellos falla en el acto en vez de propagar un valor inventado. CONFIRMADO el 01/09 que hay acceso al montaje esta misma semana, asi que la tarea deja de depender de la reserva de las semanas 9 a 11.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="25.5" customHeight="1" s="22">
       <c r="A21" s="12" t="n">
         <v>18</v>
       </c>
@@ -2206,7 +2133,7 @@
       </c>
       <c r="G21" s="12" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Hecho</t>
         </is>
       </c>
       <c r="H21" s="12" t="inlineStr">
@@ -2216,11 +2143,11 @@
       </c>
       <c r="I21" s="13" t="inlineStr">
         <is>
-          <t>Depende de terceros: pedirla el lunes 24, no al final de la semana. Las semanas 9 a 11 son las unicas ventanas de laboratorio del cronograma.</t>
-        </is>
-      </c>
-    </row>
-    <row r="22" ht="25.5" customHeight="1">
+          <t>Depende de terceros: pedirla el lunes 24, no al final de la semana. Las semanas 9 a 11 son las unicas ventanas de laboratorio del cronograma. RESERVADA en la semana 7.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="25.5" customHeight="1" s="22">
       <c r="A22" s="12" t="n">
         <v>19</v>
       </c>
@@ -2249,7 +2176,7 @@
       </c>
       <c r="G22" s="12" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Hecho</t>
         </is>
       </c>
       <c r="H22" s="12" t="inlineStr">
@@ -2257,9 +2184,13 @@
           <t>28/08/2026</t>
         </is>
       </c>
-      <c r="I22" s="13" t="n"/>
-    </row>
-    <row r="23" ht="25.5" customHeight="1">
+      <c r="I22" s="13" t="inlineStr">
+        <is>
+          <t>Hechas. Las figuras salen de la bateria regenerada el 30/08 con el codigo al dia (tarea 71), no de corridas viejas.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="25.5" customHeight="1" s="22">
       <c r="A23" s="12" t="n">
         <v>20</v>
       </c>
@@ -2288,7 +2219,7 @@
       </c>
       <c r="G23" s="12" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Hecho</t>
         </is>
       </c>
       <c r="H23" s="12" t="inlineStr">
@@ -2296,9 +2227,13 @@
           <t>28/08/2026</t>
         </is>
       </c>
-      <c r="I23" s="13" t="n"/>
-    </row>
-    <row r="24" ht="25.5" customHeight="1">
+      <c r="I23" s="13" t="inlineStr">
+        <is>
+          <t>Hecha antes del avance del 31/08.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="25.5" customHeight="1" s="22">
       <c r="A24" s="15" t="n">
         <v>21</v>
       </c>
@@ -2327,7 +2262,7 @@
       </c>
       <c r="G24" s="15" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Hecho</t>
         </is>
       </c>
       <c r="H24" s="15" t="inlineStr">
@@ -2335,9 +2270,13 @@
           <t>31/08/2026</t>
         </is>
       </c>
-      <c r="I24" s="16" t="n"/>
-    </row>
-    <row r="25" ht="25.5" customHeight="1">
+      <c r="I24" s="16" t="inlineStr">
+        <is>
+          <t>PRESENTADA el 31/08. Sin observaciones que cambien el plan: las fechas de los hitos y el arranque de la Fase 2 el 14/09 quedan como estaban. Ver tarea 22.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="25.5" customHeight="1" s="22">
       <c r="A25" s="15" t="n">
         <v>22</v>
       </c>
@@ -2366,7 +2305,7 @@
       </c>
       <c r="G25" s="15" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Hecho</t>
         </is>
       </c>
       <c r="H25" s="15" t="inlineStr">
@@ -2374,9 +2313,13 @@
           <t>31/08/2026</t>
         </is>
       </c>
-      <c r="I25" s="16" t="n"/>
-    </row>
-    <row r="26" ht="25.5" customHeight="1">
+      <c r="I25" s="16" t="inlineStr">
+        <is>
+          <t>CERRADA el 01/09. La retroalimentacion del avance 1 no trajo ajustes al cronograma, asi que el plan sigue vigente sin cambios. Lo que decide el arranque de la Fase 2 no es esta retroalimentacion sino la tarea 17, que sigue vencida.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="25.5" customHeight="1" s="22">
       <c r="A26" s="12" t="n">
         <v>23</v>
       </c>
@@ -2417,7 +2360,7 @@
       </c>
       <c r="I26" s="13" t="n"/>
     </row>
-    <row r="27" ht="25.5" customHeight="1">
+    <row r="27" ht="25.5" customHeight="1" s="22">
       <c r="A27" s="12" t="n">
         <v>24</v>
       </c>
@@ -2460,7 +2403,7 @@
         </is>
       </c>
     </row>
-    <row r="28" ht="25.5" customHeight="1">
+    <row r="28" ht="25.5" customHeight="1" s="22">
       <c r="A28" s="12" t="n">
         <v>25</v>
       </c>
@@ -2503,7 +2446,7 @@
         </is>
       </c>
     </row>
-    <row r="29" ht="25.5" customHeight="1">
+    <row r="29" ht="25.5" customHeight="1" s="22">
       <c r="A29" s="12" t="n">
         <v>26</v>
       </c>
@@ -2542,11 +2485,11 @@
       </c>
       <c r="I29" s="13" t="inlineStr">
         <is>
-          <t>Empezada por su mitad general: CamposT/retropropagacion.py (tarea 64) ya reconstruye sobre un barrido de z con los tres propagadores del paquete, pero asume iluminacion colimada. Falta lo especifico de DLHM: la fuente puntual divergente (magnificacion M = L/z y distancia efectiva, tarea 24) y el cuarto propagador.</t>
-        </is>
-      </c>
-    </row>
-    <row r="30" ht="25.5" customHeight="1">
+          <t>Empezada por su mitad general: CamposT/retropropagacion.py (tarea 64) ya reconstruye sobre un barrido de z con los tres propagadores del paquete, pero asume iluminacion colimada. Al 31/08 se suma scripts/retro_holograma.py (tarea 67), que retropropaga un holograma ya registrado llamando a pipeline.propagar(), con los tres propagadores sobre el mismo dato y la misma z. Falta lo especifico de DLHM: la fuente puntual divergente (magnificacion M = L/z y distancia efectiva, tarea 24) y el cuarto propagador.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="25.5" customHeight="1" s="22">
       <c r="A30" s="12" t="n">
         <v>27</v>
       </c>
@@ -2589,7 +2532,7 @@
         </is>
       </c>
     </row>
-    <row r="31" ht="25.5" customHeight="1">
+    <row r="31" ht="25.5" customHeight="1" s="22">
       <c r="A31" s="12" t="n">
         <v>28</v>
       </c>
@@ -2628,7 +2571,7 @@
       </c>
       <c r="I31" s="13" t="n"/>
     </row>
-    <row r="32" ht="25.5" customHeight="1">
+    <row r="32" ht="25.5" customHeight="1" s="22">
       <c r="A32" s="12" t="n">
         <v>29</v>
       </c>
@@ -2667,7 +2610,7 @@
       </c>
       <c r="I32" s="13" t="n"/>
     </row>
-    <row r="33" ht="25.5" customHeight="1">
+    <row r="33" ht="25.5" customHeight="1" s="22">
       <c r="A33" s="12" t="n">
         <v>30</v>
       </c>
@@ -2706,7 +2649,7 @@
       </c>
       <c r="I33" s="13" t="n"/>
     </row>
-    <row r="34" ht="25.5" customHeight="1">
+    <row r="34" ht="25.5" customHeight="1" s="22">
       <c r="A34" s="12" t="n">
         <v>31</v>
       </c>
@@ -2749,7 +2692,7 @@
         </is>
       </c>
     </row>
-    <row r="35" ht="25.5" customHeight="1">
+    <row r="35" ht="25.5" customHeight="1" s="22">
       <c r="A35" s="12" t="n">
         <v>32</v>
       </c>
@@ -2792,7 +2735,7 @@
         </is>
       </c>
     </row>
-    <row r="36" ht="25.5" customHeight="1">
+    <row r="36" ht="25.5" customHeight="1" s="22">
       <c r="A36" s="12" t="n">
         <v>33</v>
       </c>
@@ -2831,7 +2774,7 @@
       </c>
       <c r="I36" s="13" t="n"/>
     </row>
-    <row r="37" ht="25.5" customHeight="1">
+    <row r="37" ht="25.5" customHeight="1" s="22">
       <c r="A37" s="12" t="n">
         <v>34</v>
       </c>
@@ -2870,7 +2813,7 @@
       </c>
       <c r="I37" s="13" t="n"/>
     </row>
-    <row r="38" ht="25.5" customHeight="1">
+    <row r="38" ht="25.5" customHeight="1" s="22">
       <c r="A38" s="12" t="n">
         <v>35</v>
       </c>
@@ -2909,7 +2852,7 @@
       </c>
       <c r="I38" s="13" t="n"/>
     </row>
-    <row r="39" ht="25.5" customHeight="1">
+    <row r="39" ht="25.5" customHeight="1" s="22">
       <c r="A39" s="12" t="n">
         <v>36</v>
       </c>
@@ -2948,7 +2891,7 @@
       </c>
       <c r="I39" s="13" t="n"/>
     </row>
-    <row r="40" ht="25.5" customHeight="1">
+    <row r="40" ht="25.5" customHeight="1" s="22">
       <c r="A40" s="12" t="n">
         <v>37</v>
       </c>
@@ -2987,7 +2930,7 @@
       </c>
       <c r="I40" s="13" t="n"/>
     </row>
-    <row r="41" ht="25.5" customHeight="1">
+    <row r="41" ht="25.5" customHeight="1" s="22">
       <c r="A41" s="12" t="n">
         <v>38</v>
       </c>
@@ -3026,7 +2969,7 @@
       </c>
       <c r="I41" s="13" t="n"/>
     </row>
-    <row r="42" ht="25.5" customHeight="1">
+    <row r="42" ht="25.5" customHeight="1" s="22">
       <c r="A42" s="12" t="n">
         <v>39</v>
       </c>
@@ -3065,7 +3008,7 @@
       </c>
       <c r="I42" s="13" t="n"/>
     </row>
-    <row r="43" ht="25.5" customHeight="1">
+    <row r="43" ht="25.5" customHeight="1" s="22">
       <c r="A43" s="12" t="n">
         <v>40</v>
       </c>
@@ -3104,7 +3047,7 @@
       </c>
       <c r="I43" s="13" t="n"/>
     </row>
-    <row r="44" ht="25.5" customHeight="1">
+    <row r="44" ht="25.5" customHeight="1" s="22">
       <c r="A44" s="12" t="n">
         <v>41</v>
       </c>
@@ -3143,7 +3086,7 @@
       </c>
       <c r="I44" s="13" t="n"/>
     </row>
-    <row r="45" ht="25.5" customHeight="1">
+    <row r="45" ht="25.5" customHeight="1" s="22">
       <c r="A45" s="12" t="n">
         <v>42</v>
       </c>
@@ -3182,7 +3125,7 @@
       </c>
       <c r="I45" s="13" t="n"/>
     </row>
-    <row r="46" ht="25.5" customHeight="1">
+    <row r="46" ht="25.5" customHeight="1" s="22">
       <c r="A46" s="12" t="n">
         <v>43</v>
       </c>
@@ -3221,7 +3164,7 @@
       </c>
       <c r="I46" s="13" t="n"/>
     </row>
-    <row r="47" ht="25.5" customHeight="1">
+    <row r="47" ht="25.5" customHeight="1" s="22">
       <c r="A47" s="12" t="n">
         <v>44</v>
       </c>
@@ -3260,7 +3203,7 @@
       </c>
       <c r="I47" s="13" t="n"/>
     </row>
-    <row r="48" ht="25.5" customHeight="1">
+    <row r="48" ht="25.5" customHeight="1" s="22">
       <c r="A48" s="12" t="n">
         <v>45</v>
       </c>
@@ -3299,7 +3242,7 @@
       </c>
       <c r="I48" s="13" t="n"/>
     </row>
-    <row r="49" ht="25.5" customHeight="1">
+    <row r="49" ht="25.5" customHeight="1" s="22">
       <c r="A49" s="12" t="n">
         <v>46</v>
       </c>
@@ -3338,7 +3281,7 @@
       </c>
       <c r="I49" s="13" t="n"/>
     </row>
-    <row r="50" ht="25.5" customHeight="1">
+    <row r="50" ht="25.5" customHeight="1" s="22">
       <c r="A50" s="12" t="n">
         <v>47</v>
       </c>
@@ -3377,7 +3320,7 @@
       </c>
       <c r="I50" s="13" t="n"/>
     </row>
-    <row r="51" ht="25.5" customHeight="1">
+    <row r="51" ht="25.5" customHeight="1" s="22">
       <c r="A51" s="15" t="n">
         <v>48</v>
       </c>
@@ -3416,7 +3359,7 @@
       </c>
       <c r="I51" s="16" t="n"/>
     </row>
-    <row r="52" ht="25.5" customHeight="1">
+    <row r="52" ht="25.5" customHeight="1" s="22">
       <c r="A52" s="12" t="n">
         <v>49</v>
       </c>
@@ -3455,7 +3398,7 @@
       </c>
       <c r="I52" s="13" t="n"/>
     </row>
-    <row r="53" ht="25.5" customHeight="1">
+    <row r="53" ht="25.5" customHeight="1" s="22">
       <c r="A53" s="12" t="n">
         <v>50</v>
       </c>
@@ -3494,7 +3437,7 @@
       </c>
       <c r="I53" s="13" t="n"/>
     </row>
-    <row r="54" ht="25.5" customHeight="1">
+    <row r="54" ht="25.5" customHeight="1" s="22">
       <c r="A54" s="15" t="n">
         <v>51</v>
       </c>
@@ -3533,7 +3476,7 @@
       </c>
       <c r="I54" s="16" t="n"/>
     </row>
-    <row r="55" ht="25.5" customHeight="1">
+    <row r="55" ht="25.5" customHeight="1" s="22">
       <c r="A55" s="12" t="n">
         <v>52</v>
       </c>
@@ -3572,7 +3515,7 @@
       </c>
       <c r="I55" s="13" t="n"/>
     </row>
-    <row r="56" ht="25.5" customHeight="1">
+    <row r="56" ht="25.5" customHeight="1" s="22">
       <c r="A56" s="12" t="n">
         <v>53</v>
       </c>
@@ -3611,7 +3554,7 @@
       </c>
       <c r="I56" s="13" t="n"/>
     </row>
-    <row r="57" ht="25.5" customHeight="1">
+    <row r="57" ht="25.5" customHeight="1" s="22">
       <c r="A57" s="12" t="n">
         <v>54</v>
       </c>
@@ -3650,7 +3593,7 @@
       </c>
       <c r="I57" s="13" t="n"/>
     </row>
-    <row r="58" ht="25.5" customHeight="1">
+    <row r="58" ht="25.5" customHeight="1" s="22">
       <c r="A58" s="12" t="n">
         <v>55</v>
       </c>
@@ -3689,7 +3632,7 @@
       </c>
       <c r="I58" s="13" t="n"/>
     </row>
-    <row r="59" ht="25.5" customHeight="1">
+    <row r="59" ht="25.5" customHeight="1" s="22">
       <c r="A59" s="15" t="n">
         <v>56</v>
       </c>
@@ -3728,7 +3671,7 @@
       </c>
       <c r="I59" s="16" t="n"/>
     </row>
-    <row r="60" ht="25.5" customHeight="1">
+    <row r="60" ht="25.5" customHeight="1" s="22">
       <c r="A60" s="12" t="n">
         <v>57</v>
       </c>
@@ -3771,7 +3714,7 @@
         </is>
       </c>
     </row>
-    <row r="61" ht="25.5" customHeight="1">
+    <row r="61" ht="25.5" customHeight="1" s="22">
       <c r="A61" s="12" t="n">
         <v>58</v>
       </c>
@@ -3814,7 +3757,7 @@
         </is>
       </c>
     </row>
-    <row r="62" ht="25.5" customHeight="1">
+    <row r="62" ht="25.5" customHeight="1" s="22">
       <c r="A62" s="12" t="n">
         <v>59</v>
       </c>
@@ -3857,7 +3800,7 @@
         </is>
       </c>
     </row>
-    <row r="63">
+    <row r="63" ht="118.8" customHeight="1" s="22">
       <c r="A63" s="12" t="n">
         <v>60</v>
       </c>
@@ -3900,7 +3843,7 @@
         </is>
       </c>
     </row>
-    <row r="64">
+    <row r="64" ht="145.2" customHeight="1" s="22">
       <c r="A64" s="12" t="n">
         <v>61</v>
       </c>
@@ -3943,7 +3886,7 @@
         </is>
       </c>
     </row>
-    <row r="65">
+    <row r="65" ht="132" customHeight="1" s="22">
       <c r="A65" s="12" t="n">
         <v>62</v>
       </c>
@@ -3986,7 +3929,7 @@
         </is>
       </c>
     </row>
-    <row r="66">
+    <row r="66" ht="237.6" customHeight="1" s="22">
       <c r="A66" s="12" t="n">
         <v>63</v>
       </c>
@@ -4029,7 +3972,7 @@
         </is>
       </c>
     </row>
-    <row r="67">
+    <row r="67" ht="343.2" customHeight="1" s="22">
       <c r="A67" s="12" t="n">
         <v>64</v>
       </c>
@@ -4072,7 +4015,7 @@
         </is>
       </c>
     </row>
-    <row r="68">
+    <row r="68" ht="409.6" customHeight="1" s="22">
       <c r="A68" s="12" t="n">
         <v>65</v>
       </c>
@@ -4115,16 +4058,397 @@
         </is>
       </c>
     </row>
-    <row r="69"/>
-    <row r="70">
-      <c r="D70" t="inlineStr">
-        <is>
-          <t>Ejemplo de uso: 'En curso' mientras trabajas la tarea, 'Bloqueado' si depende de un tercero (laboratorio, asesor).</t>
+    <row r="69" ht="25.5" customHeight="1" s="22">
+      <c r="A69" s="12" t="n">
+        <v>66</v>
+      </c>
+      <c r="B69" s="12" t="n">
+        <v>7</v>
+      </c>
+      <c r="C69" s="12" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
+      <c r="D69" s="13" t="inlineStr">
+        <is>
+          <t>Centrar la rejilla de frecuencias con fftfreq en FFT-ASM y BL-ASM</t>
+        </is>
+      </c>
+      <c r="E69" s="13" t="inlineStr">
+        <is>
+          <t>Propagadores correctos en malla impar</t>
+        </is>
+      </c>
+      <c r="F69" s="12" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="G69" s="12" t="inlineStr">
+        <is>
+          <t>Hecho</t>
+        </is>
+      </c>
+      <c r="H69" s="12" t="inlineStr">
+        <is>
+          <t>28/08/2026</t>
+        </is>
+      </c>
+      <c r="I69" s="13" t="inlineStr">
+        <is>
+          <t>Commit 93bd392. Los dos construian la rejilla como (arange(n) - n/2)/(delta*n) y la emparejaban con fftshift, que deja la componente continua en el indice n//2: esa expresion vale 0 ahi SOLO SI n ES PAR. Con n impar la rejilla queda medio paso corrida, H se evalua fuera de sitio y el campo propagado sale desplazado lambda*z*(0.5/(delta*n))/delta pixeles. Medido contra el gaussiano analitico en malla 65x65: RMS 4.2e-2 antes y 5.5e-4 despues; en 64x64 las dos rejillas coinciden hasta el ultimo bit, asi que esto NO puede mover ningun resultado anterior. El fallo era MUDO: el medio paso se aplica en la ida y otra vez en la vuelta y se cancela, asi que ninguna prueba de reversibilidad podia verlo y hubo que contrastar contra una solucion analitica. mpasm no lo tenia -construye su rejilla junto con las matrices de la DFT, sin fftshift de por medio-. Ahora frecuencias_fft(n, delta) es la unica fuente para los dos, la misma correccion va en los scripts sueltos via indices_centrados(), y hay 16 pruebas nuevas, una de ellas de regresion con los dos lados fijados por monkeypatch.</t>
+        </is>
+      </c>
+    </row>
+    <row r="70" ht="25.5" customHeight="1" s="22">
+      <c r="A70" s="12" t="n">
+        <v>67</v>
+      </c>
+      <c r="B70" s="12" t="n">
+        <v>7</v>
+      </c>
+      <c r="C70" s="12" t="inlineStr">
+        <is>
+          <t>F2</t>
+        </is>
+      </c>
+      <c r="D70" s="13" t="inlineStr">
+        <is>
+          <t>Anadir retro_holograma.py: retropropagar un holograma con el propagador que elijas</t>
+        </is>
+      </c>
+      <c r="E70" s="13" t="inlineStr">
+        <is>
+          <t>Reconstruccion sobre dato ya registrado</t>
+        </is>
+      </c>
+      <c r="F70" s="12" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="G70" s="12" t="inlineStr">
+        <is>
+          <t>Hecho</t>
+        </is>
+      </c>
+      <c r="H70" s="12" t="inlineStr">
+        <is>
+          <t>28/08/2026</t>
+        </is>
+      </c>
+      <c r="I70" s="13" t="inlineStr">
+        <is>
+          <t>Commit 4939608. Los otros retro_*.py demuestran un propagador cada uno sobre un objeto sintetico y hacen la ida y la vuelta; este no demuestra ninguno: recibe un holograma que ya existe y lo lleva al plano del objeto llamando a CamposT.pipeline.propagar(), en vez de cargar una cuarta copia de los propagadores. USAR_ANGULAR / USAR_BLAS / USAR_MPASM: varios en True se comparan en la misma figura, sobre el mismo dato y la misma z, que es la unica forma honesta de compararlos. RECORTAR abre la imagen y deja arrastrar la ventana con el raton; imprime el radio del cono de difraccion z*tan(theta)/delta -534 px con 633 nm, 3.45 um y z = 20 mm- y avisa cuando la ROI se queda corta, pero recorta igual: es una decision del que mira, no una guarda. La extension decide la entrada: imagen -&gt; intensidad medida, campo = sqrt(I), con la gemela encima; .npy -&gt; campo complejo, y ahi la vuelta deshace la ida exactamente. GAMMA_GUARDADO deshace la gamma del PNG antes de la raiz: con los 0.6 de resultados/campos/ no solo falsea el contraste, mueve la distancia a la que enfoca la reconstruccion. Es el script con el que se atacaran los hologramas reales de la semana 11.</t>
+        </is>
+      </c>
+    </row>
+    <row r="71" ht="25.5" customHeight="1" s="22">
+      <c r="A71" s="12" t="n">
+        <v>68</v>
+      </c>
+      <c r="B71" s="12" t="n">
+        <v>7</v>
+      </c>
+      <c r="C71" s="12" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
+      <c r="D71" s="13" t="inlineStr">
+        <is>
+          <t>Anadir el modo mixto de objeto: amplitud y fase acopladas</t>
+        </is>
+      </c>
+      <c r="E71" s="13" t="inlineStr">
+        <is>
+          <t>Objeto que absorbe y retarda</t>
+        </is>
+      </c>
+      <c r="F71" s="12" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="G71" s="12" t="inlineStr">
+        <is>
+          <t>Hecho</t>
+        </is>
+      </c>
+      <c r="H71" s="12" t="inlineStr">
+        <is>
+          <t>28/08/2026</t>
+        </is>
+      </c>
+      <c r="I71" s="13" t="inlineStr">
+        <is>
+          <t>Commit 66efe91. load_field tenia los dos extremos -'amplitud' con U0 = t y fase 0, y 'fase' con U0 = exp(i*d*t) y amplitud plana- pero no el caso general, que es el que modela una muestra real: U0 = t*exp(i*phase_depth*t). LA TRAMPA, escrita en el docstring y fijada en test_objeto_mixto.py: sobre un objeto BINARIO el modo es degenerado y phase_depth NO HACE NADA, porque queda 0 donde t=0 y exp(i*phase_depth) donde t=1, o sea el campo entero por una constante de modulo 1: una fase GLOBAL, que se cancela en |U|^2 y conmuta con la propagacion. Medido sobre usaf_like barriendo phase_depth de 0 a 2pi: contraste del holograma 2.129 y correlacion de la reconstruccion 0.725, las dos constantes hasta el ultimo decimal. usaf_like es binario, asi que el modo necesita escala de grises: resultados/campos/entrada_gris.png, el USAF suavizado a 219 niveles. scripts/mi_prueba.py exploro el parametro en linea (commit 1c335ba) y al 31/08 esta borrado en el arbol de trabajo, sin commitear.</t>
+        </is>
+      </c>
+    </row>
+    <row r="72" ht="25.5" customHeight="1" s="22">
+      <c r="A72" s="12" t="n">
+        <v>69</v>
+      </c>
+      <c r="B72" s="12" t="n">
+        <v>7</v>
+      </c>
+      <c r="C72" s="12" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
+      <c r="D72" s="13" t="inlineStr">
+        <is>
+          <t>Quitar la gamma del guardado: los barridos pintaban amplitud etiquetada como intensidad</t>
+        </is>
+      </c>
+      <c r="E72" s="13" t="inlineStr">
+        <is>
+          <t>Pilas de foco en intensidad de verdad</t>
+        </is>
+      </c>
+      <c r="F72" s="12" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="G72" s="12" t="inlineStr">
+        <is>
+          <t>Hecho</t>
+        </is>
+      </c>
+      <c r="H72" s="12" t="inlineStr">
+        <is>
+          <t>28/08/2026</t>
+        </is>
+      </c>
+      <c r="I72" s="13" t="inlineStr">
+        <is>
+          <t>Commits 30cfabb (spec) y 8733a19. guardar_png aplicaba gamma 0.5, justificada en su docstring para que la pila y la figura del mismo barrido se parecieran. Pero los paneles aplicaban la misma gamma, y (|U|^2/max)^0.5 = |U|/sqrt(max): ninguna de las dos ensenaba intensidad, las dos ensenaban AMPLITUD con la etiqueta |U|^2 puesta. Medido sobre la reconstruccion a 150 mm: nivel medio 35 sin gamma frente a 89 con ella. La division por el maximo se queda -un PNG de 8 bits no admite floats- porque es lineal y no cambia la relacion entre valores. La prueba de la gamma se reescribio en DOS, una de lo que si se escribe y otra de lo que no: sin la segunda, quien reintrodujera el **0.5 veria fallar una prueba que habla de intensidad y podria pensar que la que sobra es la prueba.</t>
+        </is>
+      </c>
+    </row>
+    <row r="73" ht="25.5" customHeight="1" s="22">
+      <c r="A73" s="12" t="n">
+        <v>70</v>
+      </c>
+      <c r="B73" s="12" t="n">
+        <v>7</v>
+      </c>
+      <c r="C73" s="12" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
+      <c r="D73" s="13" t="inlineStr">
+        <is>
+          <t>Unificar la serie retro_*: mismo esqueleto y misma figura de 3x3</t>
+        </is>
+      </c>
+      <c r="E73" s="13" t="inlineStr">
+        <is>
+          <t>Cuatro scripts comparables entre si</t>
+        </is>
+      </c>
+      <c r="F73" s="12" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="G73" s="12" t="inlineStr">
+        <is>
+          <t>Hecho</t>
+        </is>
+      </c>
+      <c r="H73" s="12" t="inlineStr">
+        <is>
+          <t>28/08/2026</t>
+        </is>
+      </c>
+      <c r="I73" s="13" t="inlineStr">
+        <is>
+          <t>Commits 476948e y e39a2d0. retro_fft_angular baja de 830 a 571 lineas -se queda el calculo (objeto, +Z, holograma, -Z, reconstruccion) y las figuras; se van siete auxiliares, el relleno de ceros y la vuelta B- y retro_mpasm adopta el mismo esqueleto: ENTRADA, PHI_MAX y los parametros en mayuscula. La figura es de 3x3: |U|^2 SIN gamma; la fase con la opacidad pesada por amplitud, porque sin eso el 91.3 % del plano tiene |U| ~ 1.3e-16 -el 2.9e-29 % de la energia- y np.angle de esos numeros llena el panel de ruido uniforme; y el campo complejo por coloreado de dominio, tono = fase y brillo = amplitud, que es donde se ve que objeto y reconstruccion son el MISMO CAMPO y no solo la misma intensidad. El barrido lleva dos metricas independientes -nitidez y RMS de fase- y sobre el USAF a Z = 10 las dos dan 10.00 mm. Se retira retro_intensidad.py. DEUDA CERRADA el 01/09 (tarea 72): las siete citas colgadas a ese archivo -seis en los tres retro_*.py y una en mi_test.py- ahora apuntan a scripts/retro_holograma.py.</t>
+        </is>
+      </c>
+    </row>
+    <row r="74" ht="25.5" customHeight="1" s="22">
+      <c r="A74" s="12" t="n">
+        <v>71</v>
+      </c>
+      <c r="B74" s="12" t="n">
+        <v>7</v>
+      </c>
+      <c r="C74" s="12" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
+      <c r="D74" s="13" t="inlineStr">
+        <is>
+          <t>Regenerar la bateria de resultados con el codigo al dia</t>
+        </is>
+      </c>
+      <c r="E74" s="13" t="inlineStr">
+        <is>
+          <t>Figuras y tablas del avance 1</t>
+        </is>
+      </c>
+      <c r="F74" s="12" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="G74" s="12" t="inlineStr">
+        <is>
+          <t>Hecho</t>
+        </is>
+      </c>
+      <c r="H74" s="12" t="inlineStr">
+        <is>
+          <t>28/08/2026</t>
+        </is>
+      </c>
+      <c r="I74" s="13" t="inlineStr">
+        <is>
+          <t>Corrida el 30/08, despues de la rejilla centrada (tarea 66), para que lo que se ensena el 31 salga del codigo de hoy y no de corridas viejas: comparacion.py -&gt; tiempos.png, aceleracion.png, escalado_N.csv y escalado_s.csv; figura_escenario.py -&gt; escenario/; y la retropropagacion del holograma z0150 con los tres propagadores sobre 30 distancias de 10 a 150 mm -&gt; retropropagacion/z0150/. Sirve ademas de comprobacion de que el paquete corre de punta a punta despues de los cambios de la semana. CERRADO el 01/09 (tarea 72): estas salidas se sacaron del repo en bd80c2f por regenerables pero no entraron en .gitignore y reaparecian sin seguimiento; ahora resultados/ va por lista blanca.</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="12" t="n">
+        <v>72</v>
+      </c>
+      <c r="B75" s="12" t="n">
+        <v>8</v>
+      </c>
+      <c r="C75" s="12" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
+      <c r="D75" s="13" t="inlineStr">
+        <is>
+          <t>Cerrar el arbol de trabajo y las deudas abiertas de la semana 7</t>
+        </is>
+      </c>
+      <c r="E75" s="13" t="inlineStr">
+        <is>
+          <t>Repo limpio y suite mas rapida</t>
+        </is>
+      </c>
+      <c r="F75" s="12" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="G75" s="12" t="inlineStr">
+        <is>
+          <t>Hecho</t>
+        </is>
+      </c>
+      <c r="H75" s="12" t="inlineStr">
+        <is>
+          <t>04/09/2026</t>
+        </is>
+      </c>
+      <c r="I75" s="13" t="inlineStr">
+        <is>
+          <t>Cerradas las deudas que venian escritas en las notas de las tareas 9, 70 y 71. UNO: tests/mi_test.py no costaba 12.2 s de recoleccion, COLGABA pytest. Su cuerpo de modulo propaga y llama seis veces a plt.show(), el backend de esta maquina es TkAgg, y pytest lo IMPORTA en cada recoleccion porque el nombre casa con *_test.py: la recoleccion se quedaba esperando a que alguien cerrara las ventanas (medido: mas de 120 s sin volver). Movido a scripts/mi_prueba_angular.py con un docstring que dice que no es una prueba, que esta superado por retro_fft_angular.py y que de su bloque de parametros solo se leen RUTA, LAMB y DELTA. LA SUITE BAJA DE 56 s A 38.29 s, 299 casos en verde antes y despues. DOS: las siete referencias colgadas a scripts/retro_intensidad.py -retirado en el commit e39a2d0- ahora apuntan a scripts/retro_holograma.py, que es de verdad lo que prometen: reconstruir desde intensidad medida en vez de deshacer una propagacion. TRES: resultados/ pasa a lista blanca (resultados/* mas !resultados/campos/) en vez de enumerar lo regenerable, porque enumerar ya fallo una vez: bd80c2f los saco del repo sin anadirlos al .gitignore y volvieron sin seguimiento a la primera corrida. CUATRO: revertidos los Z = 150, S = 1 y la RUTA a BenchmarkTarget que estaban sin commitear en los tres retro_*.py: eran una prueba, no una decision. CERRADO TODO EN LA MISMA SESION: se retira tests/z0020.png, que entro por error en 8733a19 y no lo lee ningun test; y main, que estaba en 3ef0cfa -la reorganizacion de la semana 5, 66 archivos y 8780 lineas por detras-, avanza por fusion rapida a este trabajo y se empuja a origin, asi que el repo publico deja de estar vacio (insumo de la tarea 55). Commit cbf3587. Quedan actualizadas las notas de las tareas 9, 70 y 71, que hasta hoy describian como abiertas deudas ya cerradas.</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="12" t="n">
+        <v>73</v>
+      </c>
+      <c r="B76" s="12" t="n">
+        <v>8</v>
+      </c>
+      <c r="C76" s="12" t="inlineStr">
+        <is>
+          <t>F3</t>
+        </is>
+      </c>
+      <c r="D76" s="13" t="inlineStr">
+        <is>
+          <t>Preparar la hoja de parametros y el modulo que recibira las medidas</t>
+        </is>
+      </c>
+      <c r="E76" s="13" t="inlineStr">
+        <is>
+          <t>Checklist de laboratorio + CamposT/montaje.py</t>
+        </is>
+      </c>
+      <c r="F76" s="12" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="G76" s="12" t="inlineStr">
+        <is>
+          <t>Hecho</t>
+        </is>
+      </c>
+      <c r="H76" s="12" t="inlineStr">
+        <is>
+          <t>04/09/2026</t>
+        </is>
+      </c>
+      <c r="I76" s="13" t="inlineStr">
+        <is>
+          <t>Preparado el entregable de la tarea 17 antes de la visita al laboratorio, para que la media jornada rinda y no haga falta una segunda. DOS PIEZAS. docs/hoja_parametros_montaje.md es el checklist que se lleva en la mano: cada magnitud con sus unidades, la conversion a milimetros, por que la necesita el codigo, y tres avisos que salen de fallos ya medidos -que delta_x y delta_y se anoten por separado aunque parezcan iguales, porque Kf va por eje desde la tarea 61; que el rango alcanzable de z define la malla del barrido de la tarea 29; y que hay que preguntar si la camara aplica gamma, porque la tarea 69 midio que la gamma MUEVE la distancia a la que enfoca la reconstruccion, con un metodo para averiguarlo alli mismo si no consta: dos exposiciones conocidas, y si es lineal el nivel medio se duplica-. CamposT/montaje.py es el destino de los numeros, con TABLA1 y MONTAJE SEPARADOS. HALLAZGO QUE LO MOTIVA: el repo tenia TRES longitudes de onda conviviendo -632.8 nm en figura_escenario.py y exactitud.py, que es la Tabla 1 y esta bien; 633 nm en los cuatro retro_*.py; y 405 nm en comparacion.py y mi_holograma.py-. Entre 633 y 405 hay un 56 %, y lambda entra en z_lim, en Kf, en el radio del cono de difraccion y en la distancia de enfoque. DELTA = 3.45e-3 estaba repetido en siete archivos, sin verificar. Un parametro sin medir NO vale un numero: vale el centinela SinMedir, que revienta con ParametroSinMedir en cuanto entra en una cuenta -multiplicar, dividir, potencia, float(), int(), numpy y las propiedades derivadas: once vias probadas- y dice que magnitud falta y como se obtiene. Es la misma decision que _comprobar_ventana() y que el endurecimiento de sam(): fallar fuerte antes que devolver un numero creible que luego hay que tirar. Quedan 15 parametros PENDIENTES, que son los que traera la tarea 17. figura_escenario.py y exactitud.py ya leen de TABLA1 en vez de repetir literales, con los valores identicos comprobados. 23 pruebas nuevas en tests/test_montaje.py, una de ellas de regresion sobre la DECISION y no sobre la cuenta: falla si alguien rellena un hueco con un valor plausible mientras tanto. Suite de 299 a 322 en verde. PENDIENTE A PROPOSITO: retro_holograma.py y mi_holograma.py, que son los que atacaran hologramas reales, todavia no leen de MONTAJE. Conectarlos hoy los romperia -sus parametros estan sin medir- y son las dos piezas con las que se prueba antes de la semana 11; se conectan cuando vuelvan los numeros. comparacion.py se queda con su lambda propia: es un benchmark de tiempos y el tiempo no depende de lambda.</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="12" t="n">
+        <v>74</v>
+      </c>
+      <c r="B77" s="12" t="inlineStr">
+        <is>
+          <t>Receso</t>
+        </is>
+      </c>
+      <c r="C77" s="12" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
+      <c r="D77" s="13" t="inlineStr">
+        <is>
+          <t>Anadir soporte de GPU a los cuatro barridos mi_prueba_*</t>
+        </is>
+      </c>
+      <c r="E77" s="13" t="inlineStr">
+        <is>
+          <t>Los cuatro scripts corriendo en CPU y GPU + suite de paridad</t>
+        </is>
+      </c>
+      <c r="F77" s="12" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="G77" s="12" t="inlineStr">
+        <is>
+          <t>Hecho</t>
+        </is>
+      </c>
+      <c r="H77" s="12" t="inlineStr">
+        <is>
+          <t>11/09/2026</t>
+        </is>
+      </c>
+      <c r="I77" s="13" t="inlineStr">
+        <is>
+          <t>Hecha el 08/09, en la semana de receso. Los cuatro barridos puntuados de scripts/mi_prueba_*.py aceptan ahora DISPOSITIVO -auto, cpu o gpu- y DTYPE, con la politica de CamposT.backend: complex64 en GPU, complex128 en CPU, y las FASES siempre en float64. DE DONDE SALE EL DISENO: blas y mpasm ya tenian xp y dtype en la firma de su propagador y un bloque `backend` marcado y VACIO, asi que solo faltaba quien los eligiera. angular y dlhm no podian tocarse igual porque su implementacion de referencia esta copiada tal cual -angularSpectrum de pyDHM, y point_src + angular_spectrum de dlhm.py-, asi que reciben COPIA DE TRABAJO -espectro_angular, fuente_puntual- y la referencia se queda intacta. Es lo que el encabezado de esos mismos archivos manda hacer. MEDIDO sobre BenchmarkTarget 3000x4000, la misma corrida en las dos maquinas: dlhm 152.92 s -&gt; 6.33 s (x24, 25 pasos), angular 16.54 -&gt; 0.49 (x34), mpasm 45.95 -&gt; 1.67 (x28), blas 9.19 -&gt; 0.93 (x10). Las curvas del barrido salen IDENTICAS a los cuatro decimales que imprime la consola. EQUIVALENCIA contra la referencia de cada script, que ahora se imprime en cada corrida: 0.0 EXACTO en CPU/complex128 -misma aritmetica y misma biblioteca de FFT-, 6e-16 a 1.1e-12 en GPU/complex128 -cuFFT redondea distinto que pocketfft- y 2.5e-7 a 9.0e-7 en GPU/complex64. El caso de en medio es el que separa el DISPOSITIVO de la PRECISION: lo que se pierde arriba es la mantisa, no la tarjeta. La reduccion de correlacion() va en float64 aunque el campo venga en complex64: sobre 1.2e7 sumandos el error de float32 es del orden de lo que separa dos pasos del barrido, y el argmax se iria a un z equivocado. tests/test_gpu_mi_prueba.py, 54 pruebas; suite total de 360 a 414 en verde. LO QUE NO ARREGLA, y es lo importante: la tarjeta es una RTX 3050 Laptop de 4 GB, asi que con SOBREMUESTREO = None la malla que exige la geometria en dlhm sigue siendo 13312x13312 -1.42 GB POR ARRAY en complex64, y la cadena necesita varios a la vez- y NO cabe. Lo que complex64 compra es aproximadamente el DOBLE de recorte que en CPU: ~1700 px de lado contra ~1300. El callejon que documenta la tarea 27 sigue abierto, y la salida sigue siendo puntuar por nitidez. DOS COSAS QUE LAS PRUEBAS ENCONTRARON: sincronizar() no existia en los retro_*, sale de CamposT.backend, y la atribucion que se habia escrito era falsa; y la tolerancia de GPU/complex128 no podia ser 1e-12 porque dlhm da 1.1e-12. De paso, corregido el aviso de malla rectangular de blas y mpasm, que hablaba de los ejes cruzados de angularSpectrum cuando ninguno de los dos la usa: era copia-pega desde angular y contradecia al docstring del propio archivo.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A3:I62"/>
+  <autoFilter ref="A3:I77"/>
   <mergeCells count="1">
     <mergeCell ref="A1:I1"/>
   </mergeCells>
@@ -4159,20 +4483,20 @@
   <dimension ref="A1:D13"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="14.4"/>
   <cols>
-    <col width="16" customWidth="1" min="1" max="1"/>
-    <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="56" customWidth="1" min="3" max="3"/>
-    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" style="22" min="1" max="1"/>
+    <col width="12" customWidth="1" style="22" min="2" max="2"/>
+    <col width="56" customWidth="1" style="22" min="3" max="3"/>
+    <col width="18" customWidth="1" style="22" min="4" max="4"/>
   </cols>
   <sheetData>
-    <row r="1" ht="21.75" customHeight="1">
-      <c r="A1" s="22" t="inlineStr">
+    <row r="1" ht="21.75" customHeight="1" s="22">
+      <c r="A1" s="21" t="inlineStr">
         <is>
           <t>Fechas institucionales confirmadas (Directrices 2026-2)</t>
         </is>
       </c>
     </row>
-    <row r="3" ht="30" customHeight="1">
+    <row r="3" ht="30" customHeight="1" s="22">
       <c r="A3" s="8" t="inlineStr">
         <is>
           <t>Fecha</t>
@@ -4194,7 +4518,7 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="24" customHeight="1">
+    <row r="4" ht="24" customHeight="1" s="22">
       <c r="A4" s="12" t="inlineStr">
         <is>
           <t>27 de julio de 2026</t>
@@ -4216,7 +4540,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="24" customHeight="1">
+    <row r="5" ht="24" customHeight="1" s="22">
       <c r="A5" s="12" t="inlineStr">
         <is>
           <t>3 de agosto de 2026</t>
@@ -4238,7 +4562,7 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="24" customHeight="1">
+    <row r="6" ht="24" customHeight="1" s="22">
       <c r="A6" s="12" t="inlineStr">
         <is>
           <t>31 de agosto de 2026</t>
@@ -4260,7 +4584,7 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="24" customHeight="1">
+    <row r="7" ht="24" customHeight="1" s="22">
       <c r="A7" s="12" t="inlineStr">
         <is>
           <t>19 de octubre de 2026</t>
@@ -4282,7 +4606,7 @@
         </is>
       </c>
     </row>
-    <row r="8" ht="24" customHeight="1">
+    <row r="8" ht="24" customHeight="1" s="22">
       <c r="A8" s="12" t="inlineStr">
         <is>
           <t>30 de octubre de 2026</t>
@@ -4304,7 +4628,7 @@
         </is>
       </c>
     </row>
-    <row r="9" ht="24" customHeight="1">
+    <row r="9" ht="24" customHeight="1" s="22">
       <c r="A9" s="12" t="inlineStr">
         <is>
           <t>Hasta el 20 de noviembre de 2026</t>
@@ -4326,7 +4650,7 @@
         </is>
       </c>
     </row>
-    <row r="10" ht="24" customHeight="1">
+    <row r="10" ht="24" customHeight="1" s="22">
       <c r="A10" s="12" t="inlineStr">
         <is>
           <t>Hasta el 20 de noviembre de 2026</t>
@@ -4348,7 +4672,7 @@
         </is>
       </c>
     </row>
-    <row r="11" ht="24" customHeight="1">
+    <row r="11" ht="24" customHeight="1" s="22">
       <c r="A11" s="12" t="inlineStr">
         <is>
           <t>9 y 10 de diciembre de 2026</t>
@@ -4371,7 +4695,7 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="25" t="inlineStr">
+      <c r="A13" s="24" t="inlineStr">
         <is>
           <t>Nota: la Opcion 1 (con opcion a mencion de honor) exigiria entregar el informe final el 13 de octubre (semana 13) y defender antes del 6 de noviembre. Este cronograma sigue la Opcion 2.</t>
         </is>

</xml_diff>